<commit_message>
Follow the updated metric workbook: Paid Customers, SUM(Amount) revenue
The workbook was revised after the previous commit: row 13 is renamed
Paid Deals -> Paid Customers and row 14 now spells out
SUM(Amount) for paid revenue, confirming the implementation.

Renames the paid_deals KPI key and card to paid_customers so the code
matches the workbook, and drops a stray empty metrics.py at the root.
</commit_message>
<xml_diff>
--- a/数据口径.xlsx
+++ b/数据口径.xlsx
@@ -3,8 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MyProject\dashboard\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="14000" windowHeight="14120"/>
+    <workbookView windowWidth="13545" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -162,7 +167,7 @@
     <t>"Lifecycle Stage"列中值为"Customer"、"Sales Qualified Lead"并且"Original Traffic Source"列值为"Paid"开头的字符串的行数</t>
   </si>
   <si>
-    <t>Paid Deals</t>
+    <t>Paid Customers</t>
   </si>
   <si>
     <t>COUNT((Col(Lifecycle Stage) == "Customer") and Col(Original Traffic Source) == "Paid xxx")</t>
@@ -397,7 +402,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -414,26 +419,12 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
@@ -894,19 +885,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -915,131 +915,122 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1057,17 +1048,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1393,221 +1381,221 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="19.9464285714286" customWidth="1"/>
-    <col min="2" max="2" width="18.8928571428571" customWidth="1"/>
-    <col min="3" max="3" width="66.3660714285714" customWidth="1"/>
-    <col min="4" max="4" width="41.5089285714286" customWidth="1"/>
+    <col min="1" max="1" width="19.95" customWidth="1"/>
+    <col min="2" max="2" width="18.8916666666667" customWidth="1"/>
+    <col min="3" max="3" width="66.3666666666667" customWidth="1"/>
+    <col min="4" max="4" width="41.5083333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" spans="1:4">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="34" spans="1:4">
-      <c r="A2" s="10" t="s">
+    <row r="2" ht="28.5" spans="1:4">
+      <c r="A2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="17" spans="1:4">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:4">
+      <c r="A3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="51" spans="1:4">
-      <c r="A4" s="10" t="s">
+    <row r="4" ht="42.75" spans="1:4">
+      <c r="A4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" ht="51" spans="1:4">
-      <c r="A5" s="10" t="s">
+    <row r="5" ht="28.5" spans="1:4">
+      <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" ht="34" spans="1:4">
-      <c r="A6" s="10" t="s">
+    <row r="6" ht="28.5" spans="1:4">
+      <c r="A6" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" ht="17" spans="1:4">
-      <c r="A7" s="11" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" ht="17" spans="1:4">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" ht="17" spans="1:4">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:4">
+      <c r="A9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="10" ht="69" customHeight="1" spans="1:4">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="11" ht="68" spans="1:4">
-      <c r="A11" s="10" t="s">
+    <row r="11" ht="57" spans="1:4">
+      <c r="A11" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" ht="51" spans="1:4">
-      <c r="A12" s="10" t="s">
+    <row r="12" ht="57" spans="1:4">
+      <c r="A12" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" ht="51" spans="1:4">
-      <c r="A13" s="10" t="s">
+    <row r="13" ht="42.75" spans="1:4">
+      <c r="A13" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="14" ht="57" customHeight="1" spans="1:4">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="15" ht="34" spans="1:4">
-      <c r="A15" s="10" t="s">
+    <row r="15" ht="28.5" spans="1:4">
+      <c r="A15" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1622,14 +1610,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="16.8" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9.14166666666667" defaultRowHeight="14.25" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="25.8928571428571" customWidth="1"/>
-    <col min="2" max="2" width="26.0446428571429" customWidth="1"/>
-    <col min="3" max="3" width="24.9910714285714" customWidth="1"/>
+    <col min="1" max="1" width="25.8916666666667" customWidth="1"/>
+    <col min="2" max="2" width="26.0416666666667" customWidth="1"/>
+    <col min="3" max="3" width="24.9916666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="51" spans="1:3">
+    <row r="1" s="1" customFormat="1" spans="1:3">
       <c r="A1" s="2" t="s">
         <v>50</v>
       </c>
@@ -1640,7 +1628,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="34" spans="1:3">
+    <row r="2" s="1" customFormat="1" spans="1:3">
       <c r="A2" s="2" t="s">
         <v>52</v>
       </c>
@@ -1651,7 +1639,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" ht="34" spans="1:3">
+    <row r="3" s="1" customFormat="1" spans="1:3">
       <c r="A3" s="2" t="s">
         <v>54</v>
       </c>
@@ -1662,7 +1650,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="34" spans="1:3">
+    <row r="4" s="1" customFormat="1" spans="1:3">
       <c r="A4" s="2" t="s">
         <v>56</v>
       </c>
@@ -1673,7 +1661,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="34" spans="1:3">
+    <row r="5" s="1" customFormat="1" spans="1:3">
       <c r="A5" s="2" t="s">
         <v>59</v>
       </c>
@@ -1684,235 +1672,235 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="51" spans="1:3">
+    <row r="6" s="1" customFormat="1" spans="1:3">
       <c r="A6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="51" spans="1:3">
-      <c r="A7" s="6" t="s">
+    <row r="7" s="1" customFormat="1" spans="1:3">
+      <c r="A7" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="68" spans="1:3">
-      <c r="A8" s="6" t="s">
+    <row r="8" s="1" customFormat="1" spans="1:3">
+      <c r="A8" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="84" spans="1:3">
+    <row r="9" s="1" customFormat="1" ht="28.5" spans="1:3">
       <c r="A9" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="17" spans="1:3">
+    <row r="10" s="1" customFormat="1" spans="1:3">
       <c r="A10" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="17" spans="1:3">
+    <row r="11" s="1" customFormat="1" spans="1:3">
       <c r="A11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="17" spans="1:3">
+    <row r="12" s="1" customFormat="1" spans="1:3">
       <c r="A12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="17" spans="1:3">
+    <row r="13" s="1" customFormat="1" spans="1:3">
       <c r="A13" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="34" spans="1:3">
+    <row r="14" s="1" customFormat="1" spans="1:3">
       <c r="A14" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="17" spans="1:3">
+    <row r="15" s="1" customFormat="1" spans="1:3">
       <c r="A15" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="17" spans="1:3">
+    <row r="16" s="1" customFormat="1" spans="1:3">
       <c r="A16" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="17" s="1" customFormat="1" spans="1:2">
       <c r="A17" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="18" s="1" customFormat="1" spans="1:2">
       <c r="A18" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="19" s="1" customFormat="1" spans="1:2">
       <c r="A19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="20" s="1" customFormat="1" spans="1:2">
       <c r="A20" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="21" s="1" customFormat="1" spans="1:2">
       <c r="A21" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="22" s="1" customFormat="1" spans="1:2">
       <c r="A22" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="23" s="1" customFormat="1" spans="1:2">
       <c r="A23" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="24" s="1" customFormat="1" spans="1:2">
       <c r="A24" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="25" s="1" customFormat="1" spans="1:2">
       <c r="A25" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="26" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="26" s="1" customFormat="1" spans="1:2">
       <c r="A26" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="27" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="27" s="1" customFormat="1" spans="1:2">
       <c r="A27" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="28" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="28" s="1" customFormat="1" spans="1:2">
       <c r="A28" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="29" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="29" s="1" customFormat="1" spans="1:2">
       <c r="A29" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="1" ht="34" spans="1:2">
+    <row r="30" s="1" customFormat="1" spans="1:2">
       <c r="A30" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="1" ht="34" spans="1:2">
+    <row r="31" s="1" customFormat="1" spans="1:2">
       <c r="A31" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="32" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="32" s="1" customFormat="1" spans="1:2">
       <c r="A32" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="33" s="1" customFormat="1" ht="17" spans="1:2">
+    <row r="33" s="1" customFormat="1" spans="1:2">
       <c r="A33" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="34" s="1" customFormat="1" ht="34" spans="1:2">
+    <row r="34" s="1" customFormat="1" spans="1:2">
       <c r="A34" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="7" t="s">
         <v>118</v>
       </c>
     </row>

</xml_diff>